<commit_message>
Add PiN by pop, step 1 hybrid  for Central_African_Republic___CAR
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Central_African_Republic___CAR/PiN_pop_step1_Central_African_Republic___CAR_1008_03PM.xlsx
+++ b/platform_PiN_output/Central_African_Republic___CAR/PiN_pop_step1_Central_African_Republic___CAR_1008_03PM.xlsx
@@ -524,16 +524,16 @@
         <v>172</v>
       </c>
       <c r="F2" t="n">
-        <v>50</v>
+        <v>45.5</v>
       </c>
       <c r="G2" t="n">
-        <v>297</v>
+        <v>271</v>
       </c>
       <c r="H2" t="n">
-        <v>6.3</v>
+        <v>10.7</v>
       </c>
       <c r="I2" t="n">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="J2" t="n">
         <v>14.7</v>
@@ -574,16 +574,16 @@
         <v>1300</v>
       </c>
       <c r="F3" t="n">
-        <v>29.3</v>
+        <v>26.2</v>
       </c>
       <c r="G3" t="n">
-        <v>626</v>
+        <v>560</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>7.1</v>
       </c>
       <c r="I3" t="n">
-        <v>85</v>
+        <v>152</v>
       </c>
       <c r="J3" t="n">
         <v>5.8</v>
@@ -624,16 +624,16 @@
         <v>1875</v>
       </c>
       <c r="F4" t="n">
-        <v>28.1</v>
+        <v>25.3</v>
       </c>
       <c r="G4" t="n">
-        <v>830</v>
+        <v>750</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="J4" t="n">
         <v>8.6</v>
@@ -674,16 +674,16 @@
         <v>81</v>
       </c>
       <c r="F5" t="n">
-        <v>40.4</v>
+        <v>32.3</v>
       </c>
       <c r="G5" t="n">
-        <v>163</v>
+        <v>130</v>
       </c>
       <c r="H5" t="n">
-        <v>3.6</v>
+        <v>11.7</v>
       </c>
       <c r="I5" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J5" t="n">
         <v>35.9</v>
@@ -724,16 +724,16 @@
         <v>2018</v>
       </c>
       <c r="F6" t="n">
-        <v>17.6</v>
+        <v>13.4</v>
       </c>
       <c r="G6" t="n">
-        <v>678</v>
+        <v>516</v>
       </c>
       <c r="H6" t="n">
-        <v>10.9</v>
+        <v>15.1</v>
       </c>
       <c r="I6" t="n">
-        <v>420</v>
+        <v>581</v>
       </c>
       <c r="J6" t="n">
         <v>19.2</v>
@@ -774,16 +774,16 @@
         <v>2346</v>
       </c>
       <c r="F7" t="n">
-        <v>16.2</v>
+        <v>12.7</v>
       </c>
       <c r="G7" t="n">
-        <v>584</v>
+        <v>455</v>
       </c>
       <c r="H7" t="n">
-        <v>4.5</v>
+        <v>8.1</v>
       </c>
       <c r="I7" t="n">
-        <v>163</v>
+        <v>292</v>
       </c>
       <c r="J7" t="n">
         <v>14</v>
@@ -799,7 +799,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -824,16 +824,16 @@
         <v>145</v>
       </c>
       <c r="F8" t="n">
-        <v>38.7</v>
+        <v>18.1</v>
       </c>
       <c r="G8" t="n">
-        <v>170</v>
+        <v>80</v>
       </c>
       <c r="H8" t="n">
-        <v>9.699999999999999</v>
+        <v>30.4</v>
       </c>
       <c r="I8" t="n">
-        <v>43</v>
+        <v>133</v>
       </c>
       <c r="J8" t="n">
         <v>18.7</v>
@@ -874,16 +874,16 @@
         <v>537</v>
       </c>
       <c r="F9" t="n">
-        <v>33.9</v>
+        <v>12.2</v>
       </c>
       <c r="G9" t="n">
-        <v>431</v>
+        <v>156</v>
       </c>
       <c r="H9" t="n">
-        <v>10.6</v>
+        <v>32.2</v>
       </c>
       <c r="I9" t="n">
-        <v>134</v>
+        <v>410</v>
       </c>
       <c r="J9" t="n">
         <v>13.3</v>
@@ -924,16 +924,16 @@
         <v>2191</v>
       </c>
       <c r="F10" t="n">
-        <v>53.7</v>
+        <v>48.5</v>
       </c>
       <c r="G10" t="n">
-        <v>3327</v>
+        <v>3002</v>
       </c>
       <c r="H10" t="n">
-        <v>7.9</v>
+        <v>13.1</v>
       </c>
       <c r="I10" t="n">
-        <v>487</v>
+        <v>811</v>
       </c>
       <c r="J10" t="n">
         <v>3.1</v>
@@ -974,16 +974,16 @@
         <v>1316</v>
       </c>
       <c r="F11" t="n">
-        <v>37.7</v>
+        <v>34.5</v>
       </c>
       <c r="G11" t="n">
-        <v>1149</v>
+        <v>1051</v>
       </c>
       <c r="H11" t="n">
-        <v>5.2</v>
+        <v>8.4</v>
       </c>
       <c r="I11" t="n">
-        <v>157</v>
+        <v>255</v>
       </c>
       <c r="J11" t="n">
         <v>13.9</v>
@@ -999,7 +999,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1024,16 +1024,16 @@
         <v>1214</v>
       </c>
       <c r="F12" t="n">
-        <v>35.9</v>
+        <v>29.6</v>
       </c>
       <c r="G12" t="n">
-        <v>741</v>
+        <v>611</v>
       </c>
       <c r="H12" t="n">
-        <v>1.9</v>
+        <v>8.1</v>
       </c>
       <c r="I12" t="n">
-        <v>38</v>
+        <v>168</v>
       </c>
       <c r="J12" t="n">
         <v>3.3</v>
@@ -1074,16 +1074,16 @@
         <v>1070</v>
       </c>
       <c r="F13" t="n">
-        <v>33.9</v>
+        <v>31.5</v>
       </c>
       <c r="G13" t="n">
-        <v>704</v>
+        <v>654</v>
       </c>
       <c r="H13" t="n">
-        <v>2.8</v>
+        <v>5.2</v>
       </c>
       <c r="I13" t="n">
-        <v>57</v>
+        <v>108</v>
       </c>
       <c r="J13" t="n">
         <v>11.8</v>
@@ -1124,16 +1124,16 @@
         <v>6214</v>
       </c>
       <c r="F14" t="n">
-        <v>20.6</v>
+        <v>20.2</v>
       </c>
       <c r="G14" t="n">
-        <v>1931</v>
+        <v>1889</v>
       </c>
       <c r="H14" t="n">
-        <v>2.2</v>
+        <v>2.7</v>
       </c>
       <c r="I14" t="n">
-        <v>210</v>
+        <v>252</v>
       </c>
       <c r="J14" t="n">
         <v>10.8</v>
@@ -1174,16 +1174,16 @@
         <v>2366</v>
       </c>
       <c r="F15" t="n">
-        <v>23.2</v>
+        <v>13.8</v>
       </c>
       <c r="G15" t="n">
-        <v>1142</v>
+        <v>680</v>
       </c>
       <c r="H15" t="n">
-        <v>8.300000000000001</v>
+        <v>17.7</v>
       </c>
       <c r="I15" t="n">
-        <v>408</v>
+        <v>870</v>
       </c>
       <c r="J15" t="n">
         <v>20.4</v>
@@ -1224,16 +1224,16 @@
         <v>1464</v>
       </c>
       <c r="F16" t="n">
-        <v>39.4</v>
+        <v>27.5</v>
       </c>
       <c r="G16" t="n">
-        <v>1685</v>
+        <v>1174</v>
       </c>
       <c r="H16" t="n">
-        <v>2.8</v>
+        <v>14.7</v>
       </c>
       <c r="I16" t="n">
-        <v>119</v>
+        <v>630</v>
       </c>
       <c r="J16" t="n">
         <v>23.5</v>
@@ -1274,16 +1274,16 @@
         <v>391</v>
       </c>
       <c r="F17" t="n">
-        <v>40.6</v>
+        <v>26.1</v>
       </c>
       <c r="G17" t="n">
-        <v>438</v>
+        <v>282</v>
       </c>
       <c r="H17" t="n">
-        <v>3.4</v>
+        <v>17.9</v>
       </c>
       <c r="I17" t="n">
-        <v>37</v>
+        <v>193</v>
       </c>
       <c r="J17" t="n">
         <v>19.8</v>
@@ -1324,16 +1324,16 @@
         <v>1618</v>
       </c>
       <c r="F18" t="n">
-        <v>36.3</v>
+        <v>26.8</v>
       </c>
       <c r="G18" t="n">
-        <v>1455</v>
+        <v>1073</v>
       </c>
       <c r="H18" t="n">
-        <v>10.9</v>
+        <v>20.4</v>
       </c>
       <c r="I18" t="n">
-        <v>436</v>
+        <v>818</v>
       </c>
       <c r="J18" t="n">
         <v>12.5</v>
@@ -1374,16 +1374,16 @@
         <v>127</v>
       </c>
       <c r="F19" t="n">
-        <v>25.2</v>
+        <v>23.7</v>
       </c>
       <c r="G19" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H19" t="n">
-        <v>3.2</v>
+        <v>4.7</v>
       </c>
       <c r="I19" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J19" t="n">
         <v>11</v>
@@ -1424,16 +1424,16 @@
         <v>153</v>
       </c>
       <c r="F20" t="n">
-        <v>27.2</v>
+        <v>19.7</v>
       </c>
       <c r="G20" t="n">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="H20" t="n">
-        <v>12.9</v>
+        <v>20.4</v>
       </c>
       <c r="I20" t="n">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="J20" t="n">
         <v>14</v>
@@ -1474,16 +1474,16 @@
         <v>75</v>
       </c>
       <c r="F21" t="n">
-        <v>27.9</v>
+        <v>25.2</v>
       </c>
       <c r="G21" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H21" t="n">
-        <v>10.3</v>
+        <v>12.9</v>
       </c>
       <c r="I21" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J21" t="n">
         <v>14.1</v>
@@ -1524,16 +1524,16 @@
         <v>326</v>
       </c>
       <c r="F22" t="n">
-        <v>40.5</v>
+        <v>30.5</v>
       </c>
       <c r="G22" t="n">
-        <v>347</v>
+        <v>261</v>
       </c>
       <c r="H22" t="n">
-        <v>9.800000000000001</v>
+        <v>19.8</v>
       </c>
       <c r="I22" t="n">
-        <v>83</v>
+        <v>169</v>
       </c>
       <c r="J22" t="n">
         <v>11.6</v>
@@ -1574,16 +1574,16 @@
         <v>487</v>
       </c>
       <c r="F23" t="n">
-        <v>17.4</v>
+        <v>16</v>
       </c>
       <c r="G23" t="n">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="H23" t="n">
-        <v>3.1</v>
+        <v>4.5</v>
       </c>
       <c r="I23" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="J23" t="n">
         <v>5.6</v>
@@ -1674,16 +1674,16 @@
         <v>327</v>
       </c>
       <c r="F25" t="n">
-        <v>23.2</v>
+        <v>22.7</v>
       </c>
       <c r="G25" t="n">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="H25" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J25" t="n">
         <v>28.8</v>
@@ -1724,16 +1724,16 @@
         <v>260</v>
       </c>
       <c r="F26" t="n">
-        <v>34.4</v>
+        <v>19.2</v>
       </c>
       <c r="G26" t="n">
-        <v>575</v>
+        <v>320</v>
       </c>
       <c r="H26" t="n">
-        <v>19.5</v>
+        <v>34.7</v>
       </c>
       <c r="I26" t="n">
-        <v>325</v>
+        <v>580</v>
       </c>
       <c r="J26" t="n">
         <v>30.5</v>
@@ -1774,16 +1774,16 @@
         <v>3439</v>
       </c>
       <c r="F27" t="n">
-        <v>22.6</v>
+        <v>20.1</v>
       </c>
       <c r="G27" t="n">
-        <v>1195</v>
+        <v>1066</v>
       </c>
       <c r="H27" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="I27" t="n">
-        <v>81</v>
+        <v>210</v>
       </c>
       <c r="J27" t="n">
         <v>11</v>
@@ -1824,16 +1824,16 @@
         <v>949</v>
       </c>
       <c r="F28" t="n">
-        <v>14.9</v>
+        <v>14.5</v>
       </c>
       <c r="G28" t="n">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="H28" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="I28" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J28" t="n">
         <v>7.8</v>
@@ -1874,16 +1874,16 @@
         <v>7297</v>
       </c>
       <c r="F29" t="n">
-        <v>21.5</v>
+        <v>14.8</v>
       </c>
       <c r="G29" t="n">
-        <v>2407</v>
+        <v>1655</v>
       </c>
       <c r="H29" t="n">
-        <v>4.7</v>
+        <v>11.4</v>
       </c>
       <c r="I29" t="n">
-        <v>527</v>
+        <v>1279</v>
       </c>
       <c r="J29" t="n">
         <v>8.699999999999999</v>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1924,16 +1924,16 @@
         <v>1514</v>
       </c>
       <c r="F30" t="n">
-        <v>22.6</v>
+        <v>19.4</v>
       </c>
       <c r="G30" t="n">
-        <v>828</v>
+        <v>710</v>
       </c>
       <c r="H30" t="n">
-        <v>16.1</v>
+        <v>19.4</v>
       </c>
       <c r="I30" t="n">
-        <v>592</v>
+        <v>710</v>
       </c>
       <c r="J30" t="n">
         <v>20</v>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1974,16 +1974,16 @@
         <v>4295</v>
       </c>
       <c r="F31" t="n">
-        <v>20.1</v>
+        <v>16.8</v>
       </c>
       <c r="G31" t="n">
-        <v>1218</v>
+        <v>1015</v>
       </c>
       <c r="H31" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="I31" t="n">
-        <v>203</v>
+        <v>406</v>
       </c>
       <c r="J31" t="n">
         <v>5.6</v>
@@ -2024,16 +2024,16 @@
         <v>2478</v>
       </c>
       <c r="F32" t="n">
-        <v>27.6</v>
+        <v>26.3</v>
       </c>
       <c r="G32" t="n">
-        <v>1025</v>
+        <v>977</v>
       </c>
       <c r="H32" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="I32" t="n">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="J32" t="n">
         <v>4.5</v>
@@ -2074,16 +2074,16 @@
         <v>336</v>
       </c>
       <c r="F33" t="n">
-        <v>37.6</v>
+        <v>37.3</v>
       </c>
       <c r="G33" t="n">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J33" t="n">
         <v>1.7</v>
@@ -2124,16 +2124,16 @@
         <v>3933</v>
       </c>
       <c r="F34" t="n">
-        <v>16.1</v>
+        <v>15.5</v>
       </c>
       <c r="G34" t="n">
-        <v>911</v>
+        <v>879</v>
       </c>
       <c r="H34" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="I34" t="n">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="J34" t="n">
         <v>14.1</v>
@@ -2174,16 +2174,16 @@
         <v>358</v>
       </c>
       <c r="F35" t="n">
-        <v>47.7</v>
+        <v>42.3</v>
       </c>
       <c r="G35" t="n">
-        <v>480</v>
+        <v>425</v>
       </c>
       <c r="H35" t="n">
-        <v>5</v>
+        <v>10.4</v>
       </c>
       <c r="I35" t="n">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="J35" t="n">
         <v>11.7</v>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -2224,16 +2224,16 @@
         <v>30</v>
       </c>
       <c r="F36" t="n">
-        <v>22.9</v>
+        <v>18.6</v>
       </c>
       <c r="G36" t="n">
+        <v>11</v>
+      </c>
+      <c r="H36" t="n">
         <v>14</v>
       </c>
-      <c r="H36" t="n">
-        <v>9.699999999999999</v>
-      </c>
       <c r="I36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J36" t="n">
         <v>18.6</v>
@@ -2274,13 +2274,13 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>10.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>4.6</v>
+        <v>6.5</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -2324,16 +2324,16 @@
         <v>850</v>
       </c>
       <c r="F38" t="n">
-        <v>34.2</v>
+        <v>28.2</v>
       </c>
       <c r="G38" t="n">
-        <v>850</v>
+        <v>701</v>
       </c>
       <c r="H38" t="n">
-        <v>7.4</v>
+        <v>13.4</v>
       </c>
       <c r="I38" t="n">
-        <v>184</v>
+        <v>333</v>
       </c>
       <c r="J38" t="n">
         <v>24.2</v>
@@ -2374,13 +2374,13 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -2424,16 +2424,16 @@
         <v>1902</v>
       </c>
       <c r="F40" t="n">
-        <v>22.4</v>
+        <v>21.6</v>
       </c>
       <c r="G40" t="n">
-        <v>631</v>
+        <v>608</v>
       </c>
       <c r="H40" t="n">
-        <v>5.5</v>
+        <v>6.3</v>
       </c>
       <c r="I40" t="n">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="J40" t="n">
         <v>4.6</v>
@@ -2474,16 +2474,16 @@
         <v>3145</v>
       </c>
       <c r="F41" t="n">
-        <v>34.7</v>
+        <v>28.9</v>
       </c>
       <c r="G41" t="n">
-        <v>2244</v>
+        <v>1866</v>
       </c>
       <c r="H41" t="n">
-        <v>0.6</v>
+        <v>6.5</v>
       </c>
       <c r="I41" t="n">
-        <v>42</v>
+        <v>419</v>
       </c>
       <c r="J41" t="n">
         <v>15.9</v>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -2524,16 +2524,16 @@
         <v>1236</v>
       </c>
       <c r="F42" t="n">
-        <v>33.8</v>
+        <v>33.5</v>
       </c>
       <c r="G42" t="n">
-        <v>888</v>
+        <v>881</v>
       </c>
       <c r="H42" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="I42" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="J42" t="n">
         <v>16.5</v>
@@ -2574,16 +2574,16 @@
         <v>174</v>
       </c>
       <c r="F43" t="n">
-        <v>34.1</v>
+        <v>25.6</v>
       </c>
       <c r="G43" t="n">
-        <v>133</v>
+        <v>100</v>
       </c>
       <c r="H43" t="n">
-        <v>1.1</v>
+        <v>9.6</v>
       </c>
       <c r="I43" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="J43" t="n">
         <v>20</v>
@@ -2624,16 +2624,16 @@
         <v>768</v>
       </c>
       <c r="F44" t="n">
-        <v>19.3</v>
+        <v>19</v>
       </c>
       <c r="G44" t="n">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H44" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="I44" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="J44" t="n">
         <v>10.7</v>
@@ -2674,16 +2674,16 @@
         <v>152</v>
       </c>
       <c r="F45" t="n">
-        <v>37.2</v>
+        <v>31.8</v>
       </c>
       <c r="G45" t="n">
-        <v>211</v>
+        <v>180</v>
       </c>
       <c r="H45" t="n">
-        <v>8.5</v>
+        <v>13.9</v>
       </c>
       <c r="I45" t="n">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="J45" t="n">
         <v>27.4</v>
@@ -2724,16 +2724,16 @@
         <v>1566</v>
       </c>
       <c r="F46" t="n">
-        <v>17.4</v>
+        <v>16.7</v>
       </c>
       <c r="G46" t="n">
-        <v>404</v>
+        <v>388</v>
       </c>
       <c r="H46" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="I46" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="J46" t="n">
         <v>12.9</v>
@@ -2774,16 +2774,16 @@
         <v>1558</v>
       </c>
       <c r="F47" t="n">
-        <v>34.7</v>
+        <v>28.6</v>
       </c>
       <c r="G47" t="n">
-        <v>1039</v>
+        <v>856</v>
       </c>
       <c r="H47" t="n">
-        <v>5.6</v>
+        <v>11.7</v>
       </c>
       <c r="I47" t="n">
-        <v>168</v>
+        <v>351</v>
       </c>
       <c r="J47" t="n">
         <v>7.7</v>
@@ -2874,13 +2874,13 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>22.8</v>
+        <v>21.5</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>26.6</v>
+        <v>27.8</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -2924,16 +2924,16 @@
         <v>9856</v>
       </c>
       <c r="F50" t="n">
-        <v>37.5</v>
+        <v>10.5</v>
       </c>
       <c r="G50" t="n">
-        <v>6768</v>
+        <v>1905</v>
       </c>
       <c r="H50" t="n">
-        <v>1.1</v>
+        <v>28</v>
       </c>
       <c r="I50" t="n">
-        <v>197</v>
+        <v>5059</v>
       </c>
       <c r="J50" t="n">
         <v>6.9</v>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3060,16 +3060,16 @@
         <v>374</v>
       </c>
       <c r="F2" t="n">
-        <v>48.9</v>
+        <v>47.8</v>
       </c>
       <c r="G2" t="n">
-        <v>544</v>
+        <v>532</v>
       </c>
       <c r="H2" t="n">
-        <v>5.4</v>
+        <v>6.5</v>
       </c>
       <c r="I2" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="J2" t="n">
         <v>12</v>
@@ -3160,16 +3160,16 @@
         <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>23.1</v>
+        <v>15.4</v>
       </c>
       <c r="G4" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="H4" t="n">
-        <v>30.8</v>
+        <v>38.5</v>
       </c>
       <c r="I4" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="J4" t="n">
         <v>43.6</v>
@@ -3210,16 +3210,16 @@
         <v>402</v>
       </c>
       <c r="F5" t="n">
-        <v>13.3</v>
+        <v>11.1</v>
       </c>
       <c r="G5" t="n">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="H5" t="n">
-        <v>6.7</v>
+        <v>8.9</v>
       </c>
       <c r="I5" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="J5" t="n">
         <v>32.2</v>
@@ -3260,16 +3260,16 @@
         <v>594</v>
       </c>
       <c r="F6" t="n">
-        <v>22.5</v>
+        <v>19.4</v>
       </c>
       <c r="G6" t="n">
-        <v>265</v>
+        <v>228</v>
       </c>
       <c r="H6" t="n">
-        <v>2.3</v>
+        <v>5.4</v>
       </c>
       <c r="I6" t="n">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="J6" t="n">
         <v>24.8</v>
@@ -3310,16 +3310,16 @@
         <v>79</v>
       </c>
       <c r="F7" t="n">
-        <v>40.4</v>
+        <v>23.4</v>
       </c>
       <c r="G7" t="n">
-        <v>116</v>
+        <v>67</v>
       </c>
       <c r="H7" t="n">
-        <v>19.1</v>
+        <v>36.2</v>
       </c>
       <c r="I7" t="n">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="J7" t="n">
         <v>12.8</v>
@@ -3360,16 +3360,16 @@
         <v>211</v>
       </c>
       <c r="F8" t="n">
-        <v>32.2</v>
+        <v>18.6</v>
       </c>
       <c r="G8" t="n">
-        <v>286</v>
+        <v>166</v>
       </c>
       <c r="H8" t="n">
-        <v>16.9</v>
+        <v>30.5</v>
       </c>
       <c r="I8" t="n">
-        <v>151</v>
+        <v>271</v>
       </c>
       <c r="J8" t="n">
         <v>27.1</v>
@@ -3510,16 +3510,16 @@
         <v>875</v>
       </c>
       <c r="F11" t="n">
-        <v>41.1</v>
+        <v>17.8</v>
       </c>
       <c r="G11" t="n">
-        <v>772</v>
+        <v>335</v>
       </c>
       <c r="H11" t="n">
-        <v>5.5</v>
+        <v>28.8</v>
       </c>
       <c r="I11" t="n">
-        <v>103</v>
+        <v>541</v>
       </c>
       <c r="J11" t="n">
         <v>6.8</v>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3560,16 +3560,16 @@
         <v>1181</v>
       </c>
       <c r="F12" t="n">
-        <v>25.8</v>
+        <v>19.4</v>
       </c>
       <c r="G12" t="n">
-        <v>591</v>
+        <v>443</v>
       </c>
       <c r="H12" t="n">
-        <v>4.8</v>
+        <v>11.3</v>
       </c>
       <c r="I12" t="n">
-        <v>111</v>
+        <v>258</v>
       </c>
       <c r="J12" t="n">
         <v>17.7</v>
@@ -3660,16 +3660,16 @@
         <v>2700</v>
       </c>
       <c r="F14" t="n">
-        <v>26.7</v>
+        <v>20</v>
       </c>
       <c r="G14" t="n">
-        <v>1227</v>
+        <v>920</v>
       </c>
       <c r="H14" t="n">
-        <v>2.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>123</v>
+        <v>429</v>
       </c>
       <c r="J14" t="n">
         <v>12</v>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3710,16 +3710,16 @@
         <v>905</v>
       </c>
       <c r="F15" t="n">
-        <v>47.7</v>
+        <v>22.7</v>
       </c>
       <c r="G15" t="n">
-        <v>2111</v>
+        <v>1005</v>
       </c>
       <c r="H15" t="n">
-        <v>4.5</v>
+        <v>29.5</v>
       </c>
       <c r="I15" t="n">
-        <v>201</v>
+        <v>1307</v>
       </c>
       <c r="J15" t="n">
         <v>27.3</v>
@@ -3760,16 +3760,16 @@
         <v>173</v>
       </c>
       <c r="F16" t="n">
-        <v>25.7</v>
+        <v>18.8</v>
       </c>
       <c r="G16" t="n">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="H16" t="n">
-        <v>7.9</v>
+        <v>14.9</v>
       </c>
       <c r="I16" t="n">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="J16" t="n">
         <v>19.8</v>
@@ -3860,16 +3860,16 @@
         <v>26</v>
       </c>
       <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
         <v>15</v>
       </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>6</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
       </c>
       <c r="J18" t="n">
         <v>20</v>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3910,16 +3910,16 @@
         <v>160</v>
       </c>
       <c r="F19" t="n">
-        <v>43.8</v>
+        <v>31.2</v>
       </c>
       <c r="G19" t="n">
-        <v>184</v>
+        <v>131</v>
       </c>
       <c r="H19" t="n">
-        <v>6.9</v>
+        <v>19.4</v>
       </c>
       <c r="I19" t="n">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="J19" t="n">
         <v>11.1</v>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3960,16 +3960,16 @@
         <v>240</v>
       </c>
       <c r="F20" t="n">
-        <v>34.3</v>
+        <v>22.9</v>
       </c>
       <c r="G20" t="n">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="J20" t="n">
         <v>2.9</v>
@@ -4110,16 +4110,16 @@
         <v>257</v>
       </c>
       <c r="F23" t="n">
-        <v>19.6</v>
+        <v>17.9</v>
       </c>
       <c r="G23" t="n">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="H23" t="n">
-        <v>41.1</v>
+        <v>42.9</v>
       </c>
       <c r="I23" t="n">
-        <v>493</v>
+        <v>515</v>
       </c>
       <c r="J23" t="n">
         <v>17.9</v>
@@ -4160,16 +4160,16 @@
         <v>1296</v>
       </c>
       <c r="F24" t="n">
-        <v>29.5</v>
+        <v>29.1</v>
       </c>
       <c r="G24" t="n">
-        <v>709</v>
+        <v>698</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="I24" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="J24" t="n">
         <v>13.5</v>
@@ -4360,16 +4360,16 @@
         <v>4584</v>
       </c>
       <c r="F28" t="n">
-        <v>11.6</v>
+        <v>9.1</v>
       </c>
       <c r="G28" t="n">
-        <v>665</v>
+        <v>525</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="J28" t="n">
         <v>8.5</v>
@@ -4410,16 +4410,16 @@
         <v>1197</v>
       </c>
       <c r="F29" t="n">
-        <v>20.9</v>
+        <v>19.3</v>
       </c>
       <c r="G29" t="n">
-        <v>351</v>
+        <v>324</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J29" t="n">
         <v>7.8</v>
@@ -4510,16 +4510,16 @@
         <v>1697</v>
       </c>
       <c r="F31" t="n">
-        <v>30.8</v>
+        <v>30.1</v>
       </c>
       <c r="G31" t="n">
-        <v>1103</v>
+        <v>1078</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J31" t="n">
         <v>21.8</v>
@@ -4560,16 +4560,16 @@
         <v>173</v>
       </c>
       <c r="F32" t="n">
-        <v>31.2</v>
+        <v>25</v>
       </c>
       <c r="G32" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J32" t="n">
         <v>3.1</v>
@@ -4610,16 +4610,16 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>78.90000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="G33" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H33" t="n">
-        <v>10.5</v>
+        <v>26.3</v>
       </c>
       <c r="I33" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J33" t="n">
         <v>10.5</v>
@@ -4710,16 +4710,16 @@
         <v>712</v>
       </c>
       <c r="F35" t="n">
-        <v>20</v>
+        <v>17.4</v>
       </c>
       <c r="G35" t="n">
-        <v>375</v>
+        <v>327</v>
       </c>
       <c r="H35" t="n">
-        <v>5.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I35" t="n">
-        <v>106</v>
+        <v>154</v>
       </c>
       <c r="J35" t="n">
         <v>36.4</v>
@@ -4810,16 +4810,16 @@
         <v>336</v>
       </c>
       <c r="F37" t="n">
-        <v>19.3</v>
+        <v>12.5</v>
       </c>
       <c r="G37" t="n">
-        <v>197</v>
+        <v>128</v>
       </c>
       <c r="H37" t="n">
-        <v>1.1</v>
+        <v>8</v>
       </c>
       <c r="I37" t="n">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="J37" t="n">
         <v>46.6</v>
@@ -5110,16 +5110,16 @@
         <v>875</v>
       </c>
       <c r="F43" t="n">
-        <v>20.2</v>
+        <v>19.7</v>
       </c>
       <c r="G43" t="n">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="H43" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="I43" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="J43" t="n">
         <v>12.1</v>
@@ -5310,16 +5310,16 @@
         <v>9536</v>
       </c>
       <c r="F47" t="n">
-        <v>29.6</v>
+        <v>4.9</v>
       </c>
       <c r="G47" t="n">
-        <v>4551</v>
+        <v>759</v>
       </c>
       <c r="H47" t="n">
-        <v>2.1</v>
+        <v>26.8</v>
       </c>
       <c r="I47" t="n">
-        <v>325</v>
+        <v>4118</v>
       </c>
       <c r="J47" t="n">
         <v>6.3</v>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -5446,13 +5446,13 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>42.6</v>
+        <v>31.1</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>3.3</v>
+        <v>14.8</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -5496,16 +5496,16 @@
         <v>840</v>
       </c>
       <c r="F3" t="n">
-        <v>15.6</v>
+        <v>8.1</v>
       </c>
       <c r="G3" t="n">
-        <v>229</v>
+        <v>119</v>
       </c>
       <c r="H3" t="n">
-        <v>11</v>
+        <v>18.5</v>
       </c>
       <c r="I3" t="n">
-        <v>161</v>
+        <v>272</v>
       </c>
       <c r="J3" t="n">
         <v>16.2</v>
@@ -5546,16 +5546,16 @@
         <v>368</v>
       </c>
       <c r="F4" t="n">
-        <v>20.1</v>
+        <v>16.6</v>
       </c>
       <c r="G4" t="n">
-        <v>135</v>
+        <v>111</v>
       </c>
       <c r="H4" t="n">
-        <v>5.3</v>
+        <v>8.9</v>
       </c>
       <c r="I4" t="n">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J4" t="n">
         <v>19.5</v>
@@ -5646,16 +5646,16 @@
         <v>117</v>
       </c>
       <c r="F6" t="n">
-        <v>62.1</v>
+        <v>39.4</v>
       </c>
       <c r="G6" t="n">
-        <v>229</v>
+        <v>145</v>
       </c>
       <c r="H6" t="n">
-        <v>1.5</v>
+        <v>24.2</v>
       </c>
       <c r="I6" t="n">
-        <v>6</v>
+        <v>89</v>
       </c>
       <c r="J6" t="n">
         <v>4.5</v>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -5696,16 +5696,16 @@
         <v>432</v>
       </c>
       <c r="F7" t="n">
-        <v>29.3</v>
+        <v>20.5</v>
       </c>
       <c r="G7" t="n">
-        <v>210</v>
+        <v>147</v>
       </c>
       <c r="H7" t="n">
-        <v>3.6</v>
+        <v>12.4</v>
       </c>
       <c r="I7" t="n">
-        <v>26</v>
+        <v>89</v>
       </c>
       <c r="J7" t="n">
         <v>6.8</v>
@@ -5746,16 +5746,16 @@
         <v>315</v>
       </c>
       <c r="F8" t="n">
-        <v>34.3</v>
+        <v>29.9</v>
       </c>
       <c r="G8" t="n">
-        <v>234</v>
+        <v>203</v>
       </c>
       <c r="H8" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="I8" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="J8" t="n">
         <v>17.9</v>
@@ -5771,7 +5771,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -5796,16 +5796,16 @@
         <v>1326</v>
       </c>
       <c r="F9" t="n">
-        <v>16.1</v>
+        <v>15.1</v>
       </c>
       <c r="G9" t="n">
-        <v>278</v>
+        <v>262</v>
       </c>
       <c r="H9" t="n">
-        <v>1.8</v>
+        <v>2.8</v>
       </c>
       <c r="I9" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="J9" t="n">
         <v>5.5</v>
@@ -5846,16 +5846,16 @@
         <v>312</v>
       </c>
       <c r="F10" t="n">
-        <v>23.4</v>
+        <v>16.9</v>
       </c>
       <c r="G10" t="n">
-        <v>125</v>
+        <v>90</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J10" t="n">
         <v>18.2</v>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -5896,19 +5896,19 @@
         <v>42</v>
       </c>
       <c r="F11" t="n">
-        <v>34.4</v>
+        <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>9.4</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J11" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="K11" t="n">
         <v>17</v>
@@ -5921,7 +5921,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -5946,16 +5946,16 @@
         <v>296</v>
       </c>
       <c r="F12" t="n">
-        <v>38.2</v>
+        <v>29.2</v>
       </c>
       <c r="G12" t="n">
-        <v>280</v>
+        <v>214</v>
       </c>
       <c r="H12" t="n">
-        <v>5.6</v>
+        <v>14.6</v>
       </c>
       <c r="I12" t="n">
-        <v>41</v>
+        <v>107</v>
       </c>
       <c r="J12" t="n">
         <v>15.7</v>
@@ -5996,16 +5996,16 @@
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>45.1</v>
+        <v>27.1</v>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>3.5</v>
+        <v>21.5</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
         <v>9.5</v>
@@ -6021,7 +6021,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -6046,13 +6046,13 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>26.7</v>
+        <v>13.3</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>13.3</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -6096,16 +6096,16 @@
         <v>57</v>
       </c>
       <c r="F15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" t="n">
         <v>16</v>
       </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>11</v>
-      </c>
-      <c r="H15" t="n">
-        <v>4</v>
-      </c>
-      <c r="I15" t="n">
-        <v>3</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -6196,16 +6196,16 @@
         <v>6</v>
       </c>
       <c r="F17" t="n">
-        <v>50</v>
+        <v>14.3</v>
       </c>
       <c r="G17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>35.7</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -6246,16 +6246,16 @@
         <v>169</v>
       </c>
       <c r="F18" t="n">
-        <v>23.5</v>
+        <v>20.6</v>
       </c>
       <c r="G18" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="H18" t="n">
-        <v>2.9</v>
+        <v>5.9</v>
       </c>
       <c r="I18" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J18" t="n">
         <v>2.9</v>
@@ -6346,16 +6346,16 @@
         <v>31</v>
       </c>
       <c r="F20" t="n">
-        <v>48.4</v>
+        <v>43.5</v>
       </c>
       <c r="G20" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="H20" t="n">
-        <v>14.5</v>
+        <v>19.4</v>
       </c>
       <c r="I20" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J20" t="n">
         <v>11.3</v>
@@ -6396,16 +6396,16 @@
         <v>28</v>
       </c>
       <c r="F21" t="n">
-        <v>33.8</v>
+        <v>30.8</v>
       </c>
       <c r="G21" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H21" t="n">
-        <v>26.2</v>
+        <v>29.2</v>
       </c>
       <c r="I21" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J21" t="n">
         <v>21.5</v>
@@ -6446,16 +6446,16 @@
         <v>297</v>
       </c>
       <c r="F22" t="n">
-        <v>21.2</v>
+        <v>20.6</v>
       </c>
       <c r="G22" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H22" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J22" t="n">
         <v>12.7</v>
@@ -6496,16 +6496,16 @@
         <v>67</v>
       </c>
       <c r="F23" t="n">
-        <v>17.8</v>
+        <v>16.6</v>
       </c>
       <c r="G23" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H23" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
         <v>10.1</v>
@@ -6546,16 +6546,16 @@
         <v>1598</v>
       </c>
       <c r="F24" t="n">
-        <v>7.8</v>
+        <v>7</v>
       </c>
       <c r="G24" t="n">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="H24" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="I24" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="J24" t="n">
         <v>2.3</v>
@@ -6696,16 +6696,16 @@
         <v>876</v>
       </c>
       <c r="F27" t="n">
-        <v>26.3</v>
+        <v>24.8</v>
       </c>
       <c r="G27" t="n">
-        <v>345</v>
+        <v>326</v>
       </c>
       <c r="H27" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="I27" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="J27" t="n">
         <v>6.6</v>
@@ -6796,16 +6796,16 @@
         <v>931</v>
       </c>
       <c r="F29" t="n">
-        <v>30.8</v>
+        <v>30.5</v>
       </c>
       <c r="G29" t="n">
-        <v>592</v>
+        <v>587</v>
       </c>
       <c r="H29" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="I29" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J29" t="n">
         <v>19.7</v>
@@ -7096,16 +7096,16 @@
         <v>167</v>
       </c>
       <c r="F35" t="n">
-        <v>30.6</v>
+        <v>24.7</v>
       </c>
       <c r="G35" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="H35" t="n">
-        <v>1.2</v>
+        <v>7.1</v>
       </c>
       <c r="I35" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="J35" t="n">
         <v>20</v>
@@ -7146,13 +7146,13 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>19.2</v>
+        <v>15.4</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>5.8</v>
+        <v>9.6</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -7196,13 +7196,13 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>35.1</v>
+        <v>28.6</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -7296,16 +7296,16 @@
         <v>56</v>
       </c>
       <c r="F39" t="n">
-        <v>40.7</v>
+        <v>33.3</v>
       </c>
       <c r="G39" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="H39" t="n">
-        <v>11.9</v>
+        <v>19.2</v>
       </c>
       <c r="I39" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="J39" t="n">
         <v>16.4</v>
@@ -7396,16 +7396,16 @@
         <v>987</v>
       </c>
       <c r="F41" t="n">
-        <v>27.1</v>
+        <v>26</v>
       </c>
       <c r="G41" t="n">
-        <v>421</v>
+        <v>404</v>
       </c>
       <c r="H41" t="n">
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="I41" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="J41" t="n">
         <v>5.2</v>
@@ -7546,16 +7546,16 @@
         <v>304</v>
       </c>
       <c r="F44" t="n">
-        <v>40.2</v>
+        <v>39.2</v>
       </c>
       <c r="G44" t="n">
-        <v>848</v>
+        <v>826</v>
       </c>
       <c r="H44" t="n">
-        <v>13.4</v>
+        <v>14.4</v>
       </c>
       <c r="I44" t="n">
-        <v>283</v>
+        <v>304</v>
       </c>
       <c r="J44" t="n">
         <v>32</v>
@@ -7646,16 +7646,16 @@
         <v>900</v>
       </c>
       <c r="F46" t="n">
-        <v>24.2</v>
+        <v>9.1</v>
       </c>
       <c r="G46" t="n">
-        <v>343</v>
+        <v>129</v>
       </c>
       <c r="H46" t="n">
-        <v>1.3</v>
+        <v>16.4</v>
       </c>
       <c r="I46" t="n">
-        <v>18</v>
+        <v>232</v>
       </c>
       <c r="J46" t="n">
         <v>11</v>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -7782,16 +7782,16 @@
         <v>232</v>
       </c>
       <c r="F2" t="n">
-        <v>11.3</v>
+        <v>8</v>
       </c>
       <c r="G2" t="n">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>7.3</v>
       </c>
       <c r="I2" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="J2" t="n">
         <v>25.9</v>
@@ -7832,16 +7832,16 @@
         <v>40</v>
       </c>
       <c r="F3" t="n">
-        <v>25.5</v>
+        <v>19.6</v>
       </c>
       <c r="G3" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="H3" t="n">
-        <v>3.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="J3" t="n">
         <v>52.9</v>
@@ -7882,16 +7882,16 @@
         <v>1067</v>
       </c>
       <c r="F4" t="n">
-        <v>17.9</v>
+        <v>17.1</v>
       </c>
       <c r="G4" t="n">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="H4" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="I4" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="J4" t="n">
         <v>15.4</v>
@@ -7932,16 +7932,16 @@
         <v>58</v>
       </c>
       <c r="F5" t="n">
-        <v>17.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H5" t="n">
-        <v>15.9</v>
+        <v>24.6</v>
       </c>
       <c r="I5" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J5" t="n">
         <v>26.1</v>
@@ -7982,16 +7982,16 @@
         <v>147</v>
       </c>
       <c r="F6" t="n">
-        <v>34.4</v>
+        <v>31.2</v>
       </c>
       <c r="G6" t="n">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="H6" t="n">
-        <v>6.2</v>
+        <v>9.4</v>
       </c>
       <c r="I6" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="J6" t="n">
         <v>21.9</v>
@@ -8032,16 +8032,16 @@
         <v>1329</v>
       </c>
       <c r="F7" t="n">
-        <v>22.7</v>
+        <v>16.5</v>
       </c>
       <c r="G7" t="n">
-        <v>499</v>
+        <v>364</v>
       </c>
       <c r="H7" t="n">
-        <v>5.4</v>
+        <v>11.5</v>
       </c>
       <c r="I7" t="n">
-        <v>118</v>
+        <v>254</v>
       </c>
       <c r="J7" t="n">
         <v>11.5</v>
@@ -8057,7 +8057,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8082,16 +8082,16 @@
         <v>1580</v>
       </c>
       <c r="F8" t="n">
-        <v>28.6</v>
+        <v>27.8</v>
       </c>
       <c r="G8" t="n">
-        <v>770</v>
+        <v>750</v>
       </c>
       <c r="H8" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="I8" t="n">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="J8" t="n">
         <v>9.4</v>
@@ -8282,13 +8282,13 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>9.5</v>
+        <v>8.1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>20.1</v>
+        <v>21.5</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -8332,16 +8332,16 @@
         <v>1998</v>
       </c>
       <c r="F13" t="n">
-        <v>21.7</v>
+        <v>19.9</v>
       </c>
       <c r="G13" t="n">
-        <v>754</v>
+        <v>691</v>
       </c>
       <c r="H13" t="n">
-        <v>1.4</v>
+        <v>3.3</v>
       </c>
       <c r="I13" t="n">
-        <v>50</v>
+        <v>113</v>
       </c>
       <c r="J13" t="n">
         <v>19.2</v>
@@ -8382,16 +8382,16 @@
         <v>385</v>
       </c>
       <c r="F14" t="n">
-        <v>25.6</v>
+        <v>24.8</v>
       </c>
       <c r="G14" t="n">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="H14" t="n">
-        <v>7.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="J14" t="n">
         <v>14</v>
@@ -8432,16 +8432,16 @@
         <v>549</v>
       </c>
       <c r="F15" t="n">
-        <v>26.1</v>
+        <v>20.1</v>
       </c>
       <c r="G15" t="n">
-        <v>287</v>
+        <v>221</v>
       </c>
       <c r="H15" t="n">
-        <v>9.699999999999999</v>
+        <v>15.7</v>
       </c>
       <c r="I15" t="n">
-        <v>106</v>
+        <v>172</v>
       </c>
       <c r="J15" t="n">
         <v>14.2</v>
@@ -8482,16 +8482,16 @@
         <v>1833</v>
       </c>
       <c r="F16" t="n">
-        <v>36</v>
+        <v>34.9</v>
       </c>
       <c r="G16" t="n">
-        <v>1235</v>
+        <v>1195</v>
       </c>
       <c r="H16" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="J16" t="n">
         <v>9.300000000000001</v>
@@ -8582,16 +8582,16 @@
         <v>143</v>
       </c>
       <c r="F18" t="n">
-        <v>25.4</v>
+        <v>4.4</v>
       </c>
       <c r="G18" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="J18" t="n">
         <v>15.1</v>
@@ -8607,7 +8607,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>

</xml_diff>